<commit_message>
OD1: apply owner decisions on HANDOVER items 1-21 (SPEC v0.4)
UFIC example: real age bands (SME 9/4 bands), plan->network map from the catalogue
master table, AUH splits on, riders quotable, TPA basis final (Cover statement).
Engine: blank rider = not quoted; B2 base-only and rider split; B1 override first
and rider value over the standard mix; V5 checks riders. Scorecard: single-option
scale, panels score as their lead. Benchmark: CR #13 dimensions, add-on bridging,
same-region peers with LOW_PEERS. CR log, HANDOVER, work order WS7 (CR #17).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JyzDHDYSRDvcVc7HWpwhLX
</commit_message>
<xml_diff>
--- a/fixtures/MARKET_SYN/intake/MKT-CEDAR-2026.xlsx
+++ b/fixtures/MARKET_SYN/intake/MKT-CEDAR-2026.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="44">
   <si>
     <t>MKT-CEDAR-2026</t>
   </si>
@@ -120,6 +120,9 @@
   </si>
   <si>
     <t>20% Copayment</t>
+  </si>
+  <si>
+    <t>All members</t>
   </si>
   <si>
     <t>Optical</t>
@@ -1330,7 +1333,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A5:G6"/>
+  <dimension ref="A5:G8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="5" spans="1:7">
@@ -1377,6 +1380,52 @@
       </c>
       <c r="G6">
         <v>2900</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7">
+        <v>1000</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8">
+        <v>5000</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8">
+        <v>450</v>
       </c>
     </row>
   </sheetData>
@@ -1405,13 +1454,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
@@ -1433,13 +1482,13 @@
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" t="s">
         <v>37</v>
-      </c>
-      <c r="B8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" t="s">
-        <v>36</v>
       </c>
       <c r="D8" t="s">
         <v>12</v>
@@ -1447,13 +1496,13 @@
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
@@ -1461,13 +1510,13 @@
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1475,13 +1524,13 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
@@ -1489,13 +1538,13 @@
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
@@ -1503,13 +1552,13 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>

</xml_diff>